<commit_message>
Remove the embedded Solver model; set the constraints up by hand instead
The Solver model stored as hidden defined names produced an error dialog in
Excel rather than loading configured. Excel's tolerance for that format varies by
version, and a workbook that will not open its own optimizer is worse than one
that asks for two minutes of typing.

The solver_* names are removed. The Optimization sheet now prints the exact
settings to enter: objective $B$16 maximized, changing cells $B$5:$B$7, and four
constraints — integer on the bed counts, per-crop caps, 64 beds total, 5,760
temporary hours — plus GRG Nonlinear and the non-negative option.

The model itself is unchanged and still smooth: the temporary-worker cap remains
in its hours form, so nothing Solver differentiates contains a ROUNDUP.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTd51gZjfkNzBx3Zqk1Nsf
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -60,42 +60,6 @@
     <definedName name="PMC_TOM">'MC schedules'!$F$29</definedName>
     <definedName name="PMC_CAR">'MC schedules'!$P$29</definedName>
     <definedName name="PMC_MES">'MC schedules'!$Z$39</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">Optimization!$B$16</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_adj" localSheetId="1" hidden="1">Optimization!$B$5:$B$7</definedName>
-    <definedName name="solver_eng" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="1" hidden="1">4</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Optimization!$B$5:$B$7</definedName>
-    <definedName name="solver_rel1" localSheetId="1" hidden="1">4</definedName>
-    <definedName name="solver_rhs1" localSheetId="1" hidden="1">integer</definedName>
-    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Optimization!$B$5:$B$7</definedName>
-    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Optimization!$C$5:$C$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Optimization!$B$10</definedName>
-    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Optimization!$C$10</definedName>
-    <definedName name="solver_lhs4" localSheetId="1" hidden="1">Optimization!$B$11</definedName>
-    <definedName name="solver_rel4" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rhs4" localSheetId="1" hidden="1">Optimization!$C$11</definedName>
-    <definedName name="solver_pre" localSheetId="1" hidden="1">0.000001</definedName>
-    <definedName name="solver_tol" localSheetId="1" hidden="1">0.01</definedName>
-    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_drv" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_mni" localSheetId="1" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="1" hidden="1">0.075</definedName>
-    <definedName name="solver_nod" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_rsd" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_pop" localSheetId="1" hidden="1">100</definedName>
-    <definedName name="solver_rbv" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_time" localSheetId="1" hidden="1">2147483647</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1082,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1102,7 +1066,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The Solver model is already saved in this workbook. Open Data &gt; Solver and it loads configured — just press Solve.</t>
+          <t>Enter the Solver settings below by hand — Data &gt; Solver. Five constraints, about two minutes.</t>
         </is>
       </c>
     </row>
@@ -1122,8 +1086,6 @@
           <t>Cap</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -1458,6 +1420,193 @@
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>tick Solver Add-in.  On Mac: Tools &gt; Excel Add-ins &gt; tick Solver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Solver settings — type these into Data &gt; Solver</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Set Objective</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>$B$16</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>By Changing Variable Cells</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>$B$5:$B$7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr"/>
+      <c r="B40" s="13" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Subject to the Constraints — click Add for each</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Cell Reference</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Constraint</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>$B$5:$B$7</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>$B$5:$B$7</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>$C$5:$C$7</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>$B$10</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>$C$10</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>$B$11</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>$C$11</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Select a Solving Method: GRG Nonlinear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Tick "Make Unconstrained Variables Non-Negative".</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>For the "int" constraint: pick $B$5:$B$7, then choose "int" from the relation dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>The Constraint box fills in "integer" by itself — do not type it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>If Solver is not on the Data ribbon: File &gt; Options &gt; Add-ins &gt; Manage: Excel Add-ins &gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Go &gt; tick Solver Add-in.  Mac: Tools &gt; Excel Add-ins &gt; tick Solver.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the marginal cost charts to the workbook
Three line charts on the MC schedules sheet, one per crop, each plotting marginal
cost against that crop's price across the full schedule including the diagnostic
bed past the cap. They are the source for the figures the analysis refers to.

All 18 validation checks still pass and the workbook carries its calculated values.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6XBBzYZT5GBuHp4eeXbeU
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seanbarnes/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61709E9A-6F66-674D-A0B4-90B1D7E7D945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06224F4A-7239-614A-AD04-8904C5B5AF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="680" windowWidth="25800" windowHeight="19580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7940" yWindow="1260" windowWidth="25800" windowHeight="19580" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,12 @@
     <sheet name="Checks" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">MCSchedules!$AA$7:$AA$38</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">MCSchedules!$U$7:$U$38</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">MCSchedules!$Z$7:$Z$38</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">MCSchedules!$AA$7:$AA$38</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">MCSchedules!$U$7:$U$38</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">MCSchedules!$Z$7:$Z$38</definedName>
     <definedName name="BEDS_CARROT">Optimization!$B$6</definedName>
     <definedName name="BEDS_MESCLUN">Optimization!$B$7</definedName>
     <definedName name="BEDS_TOMATO">Optimization!$B$5</definedName>
@@ -1018,7 +1024,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf applyFont="1" numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1035,6 +1041,3569 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>tomato-mc-vs-pricing</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$A$7:$A$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1469-A64F-B975-C750F934FDE6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$F$7:$F$28</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="1">
+                  <c:v>4317.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5795.6250000000036</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6703.125</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7660.859375</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4906.2750000000051</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5585.7089062500017</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6360.7668437500033</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7243.7792796875074</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8248.586534375012</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9390.7174472031256</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>10687.588677253138</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>12158.726978841107</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>13826.017053974152</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15713.977874345364</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17850.070688251115</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>20265.042286194512</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>22993.307496844121</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>26073.375326761772</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>29548.323647694342</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>33466.327879545948</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1469-A64F-B975-C750F934FDE6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$G$7:$G$28</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>8800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-1469-A64F-B975-C750F934FDE6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="2001214463"/>
+        <c:axId val="2001214911"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2001214463"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2001214911"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2001214911"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2001214463"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>carrots-mc-vs-price</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$K$7:$K$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2D13-AC49-A41C-80AAC7862CDF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$P$7:$P$28</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="1">
+                  <c:v>1507.7083333333333</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1561.0937499999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1616.481119791667</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1673.9371744791652</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1733.530731201171</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1795.332755025227</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1859.4164233334868</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1925.8571920852646</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1994.7328640100477</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2066.1236587860258</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2140.1122852607878</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2216.7840157725441</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2296.2267626316061</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2378.5311568237667</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2463.7906289988823</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2552.1014928097429</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1670.9013431626554</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1589.1387909931072</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1638.1753169880685</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1688.9454575384007</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1741.5052455431578</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2D13-AC49-A41C-80AAC7862CDF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$Q$7:$Q$28</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2094</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-2D13-AC49-A41C-80AAC7862CDF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="2001121535"/>
+        <c:axId val="1985381695"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2001121535"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1985381695"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1985381695"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2001121535"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>mesclun-mc-vs-price</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$U$7:$U$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6A8E-E546-9D69-B8CEA0EBE2EB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$Z$7:$Z$38</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="1">
+                  <c:v>2462.03125</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2501.58203125</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2541.8743896484366</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2582.920684814454</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2624.7334694862348</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2667.3254924178127</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2710.7097013180683</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2754.8992458326466</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2799.9074805692508</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2845.7479681671139</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2892.4344824110776</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2939.9810113911262</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2988.4017607077876</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2522.5810943551696</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1983.9619249331008</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2009.5273589841818</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2035.5594348357699</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2062.0658239338081</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2089.0543165975978</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2116.532823793008</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2144.5093789313105</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2172.9921396943828</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2201.9893898860464</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2231.5095413106901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2261.5611356787776</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2292.1528465402444</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2323.2934812457679</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2354.9919829366991</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2387.2574325634341</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2420.0990509335097</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2453.5262007889978</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6A8E-E546-9D69-B8CEA0EBE2EB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>MCSchedules!$AA$7:$AA$38</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;\(\$#,##0\);\-</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2700</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-6A8E-E546-9D69-B8CEA0EBE2EB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="2001925247"/>
+        <c:axId val="2001924351"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2001925247"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2001924351"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2001924351"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2001925247"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>317500</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>622300</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EEDF97E-CB0F-599D-B8EA-4627725171F8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>412750</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>565150</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F820DDC0-6B04-BD12-D6A0-4690F32D5083}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>222250</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F30F6162-8976-118B-DCB0-D91F245AB2F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5439,6 +9008,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Make the marginal cost charts readable
Each chart plotted the bed count as a data series, which drew a flat line along
zero and left the horizontal axis numbering positions rather than beds — so the
tomato crossing appeared between beds 11 and 12 when it happens between 10 and 11.
The bed counts are now bound as category labels, the two remaining series take
their names from the schedule headers, and each chart carries axis titles and a
title that describes the chart rather than the file it was going to be saved as.

All 18 validation checks still pass and the workbook carries its calculated values.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6XBBzYZT5GBuHp4eeXbeU
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -1078,7 +1078,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>tomato-mc-vs-pricing</a:t>
+              <a:t>Tomato marginal cost against price</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1121,103 +1121,17 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>MCSchedules!$A$7:$A$28</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="22"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$F$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1469-A64F-B975-C750F934FDE6}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+                  <c:v>Marginal cost</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -1230,6 +1144,81 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$A$7:$A$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$F$7:$F$28</c:f>
@@ -1310,8 +1299,19 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$G$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Price per bed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -1324,6 +1324,81 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$A$7:$A$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$G$7:$G$28</c:f>
@@ -1425,6 +1500,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Tomato beds planted</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1475,6 +1576,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Dollars per bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -1642,7 +1769,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>carrots-mc-vs-price</a:t>
+              <a:t>Carrot marginal cost against price</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1685,103 +1812,17 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>MCSchedules!$K$7:$K$28</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="22"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$P$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2D13-AC49-A41C-80AAC7862CDF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+                  <c:v>Marginal cost</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -1794,6 +1835,81 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$K$7:$K$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$P$7:$P$28</c:f>
@@ -1874,8 +1990,19 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$Q$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Price per bed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -1888,6 +2015,81 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$K$7:$K$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$Q$7:$Q$28</c:f>
@@ -1989,6 +2191,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Carrot beds planted</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2039,6 +2267,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Dollars per bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -2206,7 +2460,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>mesclun-mc-vs-price</a:t>
+              <a:t>Mesclun marginal cost against price</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2249,133 +2503,17 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>MCSchedules!$U$7:$U$38</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="32"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$Z$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>31</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6A8E-E546-9D69-B8CEA0EBE2EB}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+                  <c:v>Marginal cost</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -2388,6 +2526,111 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$U$7:$U$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$Z$7:$Z$38</c:f>
@@ -2498,8 +2741,19 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>MCSchedules!$AA$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Price per bed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -2512,6 +2766,111 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>MCSchedules!$U$7:$U$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>MCSchedules!$AA$7:$AA$38</c:f>
@@ -2643,6 +3002,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Mesclun beds planted</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2693,6 +3078,32 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Dollars per bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">

</xml_diff>